<commit_message>
feat(calculators): wip collecting more detailed previous months for beef milk intake
</commit_message>
<xml_diff>
--- a/packages/calculators/src/modules/test/3.2-beef-enteric/3.2-beef-enteric.xlsx
+++ b/packages/calculators/src/modules/test/3.2-beef-enteric/3.2-beef-enteric.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eddiesholl/Code/aginnovationaustralia/emissions-calculators/packages/calculators/src/modules/test/3.2-beef-enteric/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:20001_{660E7225-7D1D-D746-832C-34021BECDE36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:20001_{86816E00-529F-2545-9C86-ECEE4131780F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="21000" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="21000" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="3.2.1 methane" sheetId="1" r:id="rId1"/>
@@ -85,7 +85,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1516" uniqueCount="298">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1517" uniqueCount="299">
   <si>
     <t>EFPRP</t>
   </si>
@@ -759,9 +759,6 @@
     <t>Njkl</t>
   </si>
   <si>
-    <t>LCjk=4,5</t>
-  </si>
-  <si>
     <t>FAjk=4,5</t>
   </si>
   <si>
@@ -909,12 +906,6 @@
     <t>Extended region</t>
   </si>
   <si>
-    <t>LC effective</t>
-  </si>
-  <si>
-    <t>Curent or previous season LC</t>
-  </si>
-  <si>
     <t>spring</t>
   </si>
   <si>
@@ -979,6 +970,18 @@
   </si>
   <si>
     <t>Remember this needs to calculated allowing for herd movements</t>
+  </si>
+  <si>
+    <t>LCk=5 (this)</t>
+  </si>
+  <si>
+    <t>LCk=5 (prev)</t>
+  </si>
+  <si>
+    <t>FA (this season)</t>
+  </si>
+  <si>
+    <t>FA (previous season)</t>
   </si>
 </sst>
 </file>
@@ -1173,7 +1176,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1207,7 +1210,6 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -23357,51 +23359,51 @@
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>242</v>
+      </c>
+      <c r="B1" t="s">
         <v>243</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>244</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>245</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>246</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>247</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>248</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>249</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>250</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>251</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>252</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>253</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>254</v>
-      </c>
-      <c r="M1" t="s">
-        <v>255</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A2" s="9" t="s">
+        <v>240</v>
+      </c>
+      <c r="B2" s="9" t="s">
         <v>241</v>
-      </c>
-      <c r="B2" s="9" t="s">
-        <v>242</v>
       </c>
       <c r="C2" s="9"/>
       <c r="D2" t="s">
@@ -25679,6 +25681,12 @@
       <c r="V4" t="s">
         <v>47</v>
       </c>
+      <c r="AC4" t="s">
+        <v>297</v>
+      </c>
+      <c r="AD4">
+        <v>1.3</v>
+      </c>
     </row>
     <row r="5" spans="1:30" x14ac:dyDescent="0.2">
       <c r="H5" t="s">
@@ -25711,6 +25719,12 @@
       <c r="V5" t="s">
         <v>203</v>
       </c>
+      <c r="AC5" t="s">
+        <v>298</v>
+      </c>
+      <c r="AD5">
+        <v>1.1000000000000001</v>
+      </c>
     </row>
     <row r="8" spans="1:30" x14ac:dyDescent="0.2">
       <c r="H8" t="s">
@@ -25754,9 +25768,6 @@
       <c r="J9" t="s">
         <v>214</v>
       </c>
-      <c r="K9" t="s">
-        <v>275</v>
-      </c>
       <c r="L9" t="s">
         <v>215</v>
       </c>
@@ -25784,16 +25795,16 @@
         <v>59</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>62</v>
       </c>
       <c r="G10" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="H10" s="1" t="s">
         <v>222</v>
@@ -25802,46 +25813,46 @@
         <v>223</v>
       </c>
       <c r="J10" s="1" t="s">
+        <v>295</v>
+      </c>
+      <c r="K10" s="1" t="s">
+        <v>296</v>
+      </c>
+      <c r="L10" t="s">
         <v>224</v>
       </c>
-      <c r="K10" s="33" t="s">
-        <v>274</v>
-      </c>
-      <c r="L10" t="s">
+      <c r="M10" s="1" t="s">
+        <v>269</v>
+      </c>
+      <c r="N10" t="s">
         <v>225</v>
       </c>
-      <c r="M10" s="1" t="s">
+      <c r="O10" s="1" t="s">
+        <v>268</v>
+      </c>
+      <c r="P10" t="s">
+        <v>226</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>227</v>
+      </c>
+      <c r="R10" t="s">
         <v>270</v>
       </c>
-      <c r="N10" t="s">
-        <v>226</v>
-      </c>
-      <c r="O10" s="1" t="s">
-        <v>269</v>
-      </c>
-      <c r="P10" t="s">
-        <v>227</v>
-      </c>
-      <c r="Q10" t="s">
+      <c r="S10" t="s">
         <v>228</v>
       </c>
-      <c r="R10" t="s">
-        <v>271</v>
-      </c>
-      <c r="S10" t="s">
+      <c r="T10" t="s">
         <v>229</v>
       </c>
-      <c r="T10" t="s">
+      <c r="U10" t="s">
         <v>230</v>
       </c>
-      <c r="U10" t="s">
-        <v>231</v>
-      </c>
       <c r="V10" s="31" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="AC10" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="AD10" t="s">
         <v>126</v>
@@ -25852,7 +25863,7 @@
         <v>110</v>
       </c>
       <c r="B11" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="D11" t="s">
         <v>135</v>
@@ -25887,7 +25898,7 @@
         <v>1.1000000000000001</v>
       </c>
       <c r="Q11">
-        <f>(K11 * L11) + (1 - J11 )</f>
+        <f>(J11 * $AD$4 + K11*$AD$5) + (1 - J11 )</f>
         <v>1</v>
       </c>
       <c r="S11">
@@ -25904,7 +25915,7 @@
       </c>
       <c r="V11">
         <f>SUM(U11:U50)/1000</f>
-        <v>53.861310054946088</v>
+        <v>50.285648291275933</v>
       </c>
       <c r="AC11" t="s">
         <v>127</v>
@@ -25942,7 +25953,7 @@
         <v>0.33</v>
       </c>
       <c r="Q12">
-        <f t="shared" ref="Q12:Q50" si="0">(K12 * L12) + (1 - J12 )</f>
+        <f t="shared" ref="Q12:Q50" si="0">(J12 * $AD$4 + K12*$AD$5) + (1 - J12 )</f>
         <v>1</v>
       </c>
       <c r="S12">
@@ -25954,11 +25965,11 @@
         <v>0.11493047409327001</v>
       </c>
       <c r="U12">
-        <f t="shared" ref="U12:U50" si="3">H12*T12*I12</f>
+        <f>H12*T12*I12</f>
         <v>1048.7405761010889</v>
       </c>
       <c r="AA12" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="AB12" t="s">
         <v>117</v>
@@ -26008,7 +26019,7 @@
         <v>6.4887674174999993E-2</v>
       </c>
       <c r="U13">
-        <f t="shared" si="3"/>
+        <f>H13*T13*I13</f>
         <v>473.68002147749996</v>
       </c>
       <c r="AB13" t="s">
@@ -26059,7 +26070,7 @@
         <v>8.1213770643750002E-2</v>
       </c>
       <c r="U14">
-        <f t="shared" si="3"/>
+        <f>H14*T14*I14</f>
         <v>518.7529599869531</v>
       </c>
       <c r="AB14" t="s">
@@ -26113,7 +26124,7 @@
         <v>0.25445385417851996</v>
       </c>
       <c r="U15">
-        <f t="shared" si="3"/>
+        <f>H15*T15*I15</f>
         <v>464.3782838757989</v>
       </c>
       <c r="AB15" t="s">
@@ -26167,11 +26178,11 @@
         <v>0.22126857836175012</v>
       </c>
       <c r="U16">
-        <f t="shared" si="3"/>
+        <f>H16*T16*I16</f>
         <v>1615.2606220407758</v>
       </c>
       <c r="AA16" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="AB16" t="s">
         <v>117</v>
@@ -26221,7 +26232,7 @@
         <v>0.20565665279999992</v>
       </c>
       <c r="U17">
-        <f t="shared" si="3"/>
+        <f>H17*T17*I17</f>
         <v>1313.6318697599995</v>
       </c>
       <c r="AB17" t="s">
@@ -26272,7 +26283,7 @@
         <v>0.20870311459931989</v>
       </c>
       <c r="U18">
-        <f t="shared" si="3"/>
+        <f>H18*T18*I18</f>
         <v>1142.6495524312766</v>
       </c>
       <c r="AB18" t="s">
@@ -26326,7 +26337,7 @@
         <v>0.17664036603327005</v>
       </c>
       <c r="U19">
-        <f t="shared" si="3"/>
+        <f>H19*T19*I19</f>
         <v>1611.8433400535891</v>
       </c>
       <c r="AB19" t="s">
@@ -26380,7 +26391,7 @@
         <v>0.16034523412527002</v>
       </c>
       <c r="U20">
-        <f t="shared" si="3"/>
+        <f>H20*T20*I20</f>
         <v>2633.6704705075599</v>
       </c>
     </row>
@@ -26422,7 +26433,7 @@
         <v>0.12441409099199996</v>
       </c>
       <c r="U21">
-        <f t="shared" si="3"/>
+        <f>H21*T21*I21</f>
         <v>1929.9735865133994</v>
       </c>
     </row>
@@ -26464,11 +26475,11 @@
         <v>0.12332640906971998</v>
       </c>
       <c r="U22">
-        <f t="shared" si="3"/>
+        <f>H22*T22*I22</f>
         <v>1800.5655724179114</v>
       </c>
       <c r="X22" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="AP22" t="s">
         <v>184</v>
@@ -26488,15 +26499,13 @@
         <v>150</v>
       </c>
       <c r="J23">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="K23">
-        <f>J23+J26</f>
-        <v>0.79999999999999993</v>
+        <v>0</v>
       </c>
       <c r="L23">
-        <f>$AC$12</f>
-        <v>1.3</v>
+        <v>0</v>
       </c>
       <c r="N23">
         <v>560</v>
@@ -26506,25 +26515,25 @@
       </c>
       <c r="Q23">
         <f t="shared" si="0"/>
-        <v>1.34</v>
+        <v>1</v>
       </c>
       <c r="S23">
         <f t="shared" si="1"/>
-        <v>13.927245421014002</v>
+        <v>10.3934667321</v>
       </c>
       <c r="T23">
         <f t="shared" si="2"/>
-        <v>0.28829398021498981</v>
+        <v>0.21514476135447</v>
       </c>
       <c r="U23">
-        <f t="shared" si="3"/>
-        <v>3946.0238541926733</v>
+        <f>H23*T23*I23</f>
+        <v>2944.7939210393079</v>
       </c>
       <c r="X23" t="s">
         <v>130</v>
       </c>
       <c r="Y23" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="Z23" t="s">
         <v>113</v>
@@ -26539,37 +26548,37 @@
         <v>135</v>
       </c>
       <c r="AD23" t="s">
+        <v>255</v>
+      </c>
+      <c r="AE23" t="s">
         <v>256</v>
       </c>
-      <c r="AE23" t="s">
+      <c r="AF23" t="s">
         <v>257</v>
       </c>
-      <c r="AF23" t="s">
+      <c r="AG23" t="s">
         <v>258</v>
       </c>
-      <c r="AG23" t="s">
+      <c r="AH23" t="s">
         <v>259</v>
       </c>
-      <c r="AH23" t="s">
+      <c r="AI23" t="s">
         <v>260</v>
       </c>
-      <c r="AI23" t="s">
+      <c r="AJ23" t="s">
         <v>261</v>
       </c>
-      <c r="AJ23" t="s">
+      <c r="AK23" t="s">
         <v>262</v>
       </c>
-      <c r="AK23" t="s">
+      <c r="AL23" t="s">
         <v>263</v>
       </c>
-      <c r="AL23" t="s">
+      <c r="AM23" t="s">
         <v>264</v>
       </c>
-      <c r="AM23" t="s">
-        <v>265</v>
-      </c>
       <c r="AN23" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="AP23" s="10"/>
       <c r="AQ23" s="11"/>
@@ -26602,12 +26611,10 @@
         <v>0</v>
       </c>
       <c r="K24">
-        <f>J24+J23</f>
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="L24">
-        <f>$AC$13</f>
-        <v>1.1000000000000001</v>
+        <v>0</v>
       </c>
       <c r="N24">
         <v>550</v>
@@ -26617,19 +26624,19 @@
       </c>
       <c r="Q24">
         <f t="shared" si="0"/>
-        <v>1.77</v>
+        <v>1</v>
       </c>
       <c r="S24">
         <f t="shared" si="1"/>
-        <v>14.518417920000003</v>
+        <v>8.2024960000000018</v>
       </c>
       <c r="T24">
         <f t="shared" si="2"/>
-        <v>0.30053125094400002</v>
+        <v>0.16979166720000005</v>
       </c>
       <c r="U24">
-        <f t="shared" si="3"/>
-        <v>6855.8691621600001</v>
+        <f>H24*T24*I24</f>
+        <v>3873.3724080000011</v>
       </c>
       <c r="X24" s="9" t="s">
         <v>117</v>
@@ -26684,40 +26691,40 @@
       </c>
       <c r="AP24" s="14"/>
       <c r="AQ24" s="26" t="s">
+        <v>242</v>
+      </c>
+      <c r="AR24" s="27" t="s">
         <v>243</v>
       </c>
-      <c r="AR24" s="27" t="s">
+      <c r="AS24" s="28" t="s">
         <v>244</v>
       </c>
-      <c r="AS24" s="28" t="s">
+      <c r="AT24" s="28" t="s">
         <v>245</v>
       </c>
-      <c r="AT24" s="28" t="s">
+      <c r="AU24" s="28" t="s">
         <v>246</v>
       </c>
-      <c r="AU24" s="28" t="s">
+      <c r="AV24" s="29" t="s">
         <v>247</v>
       </c>
-      <c r="AV24" s="29" t="s">
+      <c r="AW24" s="28" t="s">
         <v>248</v>
       </c>
-      <c r="AW24" s="28" t="s">
+      <c r="AX24" s="28" t="s">
         <v>249</v>
       </c>
-      <c r="AX24" s="28" t="s">
+      <c r="AY24" s="28" t="s">
         <v>250</v>
       </c>
-      <c r="AY24" s="28" t="s">
+      <c r="AZ24" s="28" t="s">
         <v>251</v>
       </c>
-      <c r="AZ24" s="28" t="s">
+      <c r="BA24" s="28" t="s">
         <v>252</v>
       </c>
-      <c r="BA24" s="28" t="s">
+      <c r="BB24" s="28" t="s">
         <v>253</v>
-      </c>
-      <c r="BB24" s="28" t="s">
-        <v>254</v>
       </c>
     </row>
     <row r="25" spans="5:54" ht="17" thickTop="1" x14ac:dyDescent="0.2">
@@ -26734,7 +26741,6 @@
         <v>0</v>
       </c>
       <c r="K25">
-        <f>J25+J24</f>
         <v>0</v>
       </c>
       <c r="L25">
@@ -26760,7 +26766,7 @@
         <v>0.158198927175</v>
       </c>
       <c r="U25">
-        <f t="shared" si="3"/>
+        <f>H25*T25*I25</f>
         <v>3464.5565051325002</v>
       </c>
       <c r="X25" s="9" t="s">
@@ -26816,7 +26822,7 @@
       </c>
       <c r="AP25" s="18"/>
       <c r="AQ25" s="14" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="AR25" s="15" t="s">
         <v>130</v>
@@ -26863,11 +26869,10 @@
         <v>200</v>
       </c>
       <c r="J26">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="K26">
-        <f>J26+K25</f>
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="L26">
         <f>$AC$14</f>
@@ -26881,19 +26886,19 @@
       </c>
       <c r="Q26">
         <f t="shared" si="0"/>
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="S26">
         <f t="shared" si="1"/>
-        <v>7.1255208038400015</v>
+        <v>7.9172453376000016</v>
       </c>
       <c r="T26">
         <f t="shared" si="2"/>
-        <v>0.14749828063948803</v>
+        <v>0.16388697848832004</v>
       </c>
       <c r="U26">
-        <f t="shared" si="3"/>
-        <v>2691.8436216706564</v>
+        <f>H26*T26*I26</f>
+        <v>2990.9373574118408</v>
       </c>
       <c r="X26" s="9" t="s">
         <v>120</v>
@@ -27001,8 +27006,7 @@
         <v>0.8</v>
       </c>
       <c r="K27">
-        <f>J27+J30</f>
-        <v>0.9</v>
+        <v>0.05</v>
       </c>
       <c r="L27">
         <f>$AC$12</f>
@@ -27016,19 +27020,19 @@
       </c>
       <c r="Q27">
         <f t="shared" si="0"/>
-        <v>1.37</v>
+        <v>1.2949999999999999</v>
       </c>
       <c r="S27">
         <f t="shared" si="1"/>
-        <v>8.3673043119719992</v>
+        <v>7.9092402073019974</v>
       </c>
       <c r="T27">
         <f t="shared" si="2"/>
-        <v>0.17320319925782038</v>
+        <v>0.16372127229115133</v>
       </c>
       <c r="U27">
-        <f t="shared" si="3"/>
-        <v>1580.4791932276109</v>
+        <f>H27*T27*I27</f>
+        <v>1493.9566096567557</v>
       </c>
       <c r="X27" s="9" t="s">
         <v>121</v>
@@ -27119,7 +27123,7 @@
     </row>
     <row r="28" spans="5:54" x14ac:dyDescent="0.2">
       <c r="E28" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="F28" t="s">
         <v>119</v>
@@ -27134,8 +27138,7 @@
         <v>0</v>
       </c>
       <c r="K28">
-        <f>J28+J27</f>
-        <v>0.8</v>
+        <v>0.78</v>
       </c>
       <c r="L28">
         <f>$AC$13</f>
@@ -27149,19 +27152,19 @@
       </c>
       <c r="Q28">
         <f t="shared" si="0"/>
-        <v>1.8800000000000001</v>
+        <v>1.8580000000000001</v>
       </c>
       <c r="S28">
         <f t="shared" si="1"/>
-        <v>9.5932826563680038</v>
+        <v>9.4810208380488028</v>
       </c>
       <c r="T28">
         <f t="shared" si="2"/>
-        <v>0.19858095098681766</v>
+        <v>0.19625713134761019</v>
       </c>
       <c r="U28">
-        <f t="shared" si="3"/>
-        <v>3442.897237733951</v>
+        <f>H28*T28*I28</f>
+        <v>3402.6080147391917</v>
       </c>
       <c r="X28" s="9" t="s">
         <v>117</v>
@@ -27264,7 +27267,6 @@
         <v>0</v>
       </c>
       <c r="K29">
-        <f>J29+J28</f>
         <v>0</v>
       </c>
       <c r="L29">
@@ -27290,7 +27292,7 @@
         <v>6.4564463903557495E-2</v>
       </c>
       <c r="U29">
-        <f t="shared" si="3"/>
+        <f>H29*T29*I29</f>
         <v>1148.8439295839262</v>
       </c>
       <c r="X29" s="9" t="s">
@@ -27394,8 +27396,7 @@
         <v>0.1</v>
       </c>
       <c r="K30">
-        <f>J30+K29</f>
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="L30">
         <f>$AC$14</f>
@@ -27409,19 +27410,19 @@
       </c>
       <c r="Q30">
         <f t="shared" si="0"/>
-        <v>0.9</v>
+        <v>1.03</v>
       </c>
       <c r="S30">
         <f t="shared" si="1"/>
-        <v>3.3315637680899997</v>
+        <v>3.8127896457029995</v>
       </c>
       <c r="T30">
         <f t="shared" si="2"/>
-        <v>6.8963369999462981E-2</v>
+        <v>7.8924745666052093E-2</v>
       </c>
       <c r="U30">
-        <f t="shared" si="3"/>
-        <v>1258.5815024901995</v>
+        <f>H30*T30*I30</f>
+        <v>1440.3766084054507</v>
       </c>
       <c r="X30" s="9" t="s">
         <v>120</v>
@@ -27529,8 +27530,7 @@
         <v>0.9</v>
       </c>
       <c r="K31">
-        <f>J31+J34</f>
-        <v>0.9</v>
+        <v>0.05</v>
       </c>
       <c r="L31">
         <f>$AC$12</f>
@@ -27544,19 +27544,19 @@
       </c>
       <c r="Q31">
         <f t="shared" si="0"/>
-        <v>1.27</v>
+        <v>1.3250000000000002</v>
       </c>
       <c r="S31">
         <f t="shared" si="1"/>
-        <v>13.199702749767001</v>
+        <v>13.771343420032503</v>
       </c>
       <c r="T31">
         <f t="shared" si="2"/>
-        <v>0.27323384692017694</v>
+        <v>0.28506680879467278</v>
       </c>
       <c r="U31">
-        <f t="shared" si="3"/>
-        <v>1246.6294265733072</v>
+        <f>H31*T31*I31</f>
+        <v>1300.6173151256944</v>
       </c>
       <c r="X31" s="9" t="s">
         <v>121</v>
@@ -27647,7 +27647,7 @@
     </row>
     <row r="32" spans="5:54" x14ac:dyDescent="0.2">
       <c r="E32" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="F32" t="s">
         <v>119</v>
@@ -27662,7 +27662,6 @@
         <v>0</v>
       </c>
       <c r="K32">
-        <f>J32+J31</f>
         <v>0.9</v>
       </c>
       <c r="L32">
@@ -27688,7 +27687,7 @@
         <v>0.33788541772800013</v>
       </c>
       <c r="U32">
-        <f t="shared" si="3"/>
+        <f>H32*T32*I32</f>
         <v>3083.2044367680014</v>
       </c>
       <c r="X32" s="9" t="s">
@@ -27792,7 +27791,6 @@
         <v>0</v>
       </c>
       <c r="K33">
-        <f>J33+J32</f>
         <v>0</v>
       </c>
       <c r="L33">
@@ -27818,7 +27816,7 @@
         <v>0.158198927175</v>
       </c>
       <c r="U33">
-        <f t="shared" si="3"/>
+        <f>H33*T33*I33</f>
         <v>1299.2086894246875</v>
       </c>
       <c r="X33" s="9" t="s">
@@ -27922,7 +27920,6 @@
         <v>0</v>
       </c>
       <c r="K34">
-        <f>J34+K33</f>
         <v>0</v>
       </c>
       <c r="L34">
@@ -27948,7 +27945,7 @@
         <v>0.16388697848832004</v>
       </c>
       <c r="U34">
-        <f t="shared" si="3"/>
+        <f>H34*T34*I34</f>
         <v>1196.3749429647364</v>
       </c>
       <c r="X34" s="9" t="s">
@@ -28069,7 +28066,7 @@
         <v>0.77</v>
       </c>
       <c r="Q35">
-        <f>(K35 * L35) + (1 - J35 )</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="S35">
@@ -28081,7 +28078,7 @@
         <v>0.19467496241126997</v>
       </c>
       <c r="U35">
-        <f t="shared" si="3"/>
+        <f>H35*T35*I35</f>
         <v>532.92270960085148</v>
       </c>
       <c r="X35" s="9" t="s">
@@ -28212,7 +28209,7 @@
         <v>0.17138540797766999</v>
       </c>
       <c r="U36">
-        <f t="shared" si="3"/>
+        <f>H36*T36*I36</f>
         <v>1094.7242934573671</v>
       </c>
       <c r="X36" s="9" t="s">
@@ -28340,7 +28337,7 @@
         <v>0.14782700226492007</v>
       </c>
       <c r="U37">
-        <f t="shared" si="3"/>
+        <f>H37*T37*I37</f>
         <v>539.56855826695823</v>
       </c>
       <c r="X37" s="9" t="s">
@@ -28468,7 +28465,7 @@
         <v>0.16034523412527002</v>
       </c>
       <c r="U38">
-        <f t="shared" si="3"/>
+        <f>H38*T38*I38</f>
         <v>292.63005227861777</v>
       </c>
       <c r="X38" s="9" t="s">
@@ -28601,7 +28598,7 @@
         <v>0.19467496241126997</v>
       </c>
       <c r="U39">
-        <f t="shared" si="3"/>
+        <f>H39*T39*I39</f>
         <v>532.92270960085148</v>
       </c>
       <c r="X39" s="9" t="s">
@@ -28693,7 +28690,7 @@
     </row>
     <row r="40" spans="5:54" x14ac:dyDescent="0.2">
       <c r="E40" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="F40" t="s">
         <v>119</v>
@@ -28732,7 +28729,7 @@
         <v>0.17138540797766999</v>
       </c>
       <c r="U40">
-        <f t="shared" si="3"/>
+        <f>H40*T40*I40</f>
         <v>1563.8918477962386</v>
       </c>
       <c r="X40" s="9" t="s">
@@ -28860,7 +28857,7 @@
         <v>0.14782700226492007</v>
       </c>
       <c r="U41">
-        <f t="shared" si="3"/>
+        <f>H41*T41*I41</f>
         <v>539.56855826695823</v>
       </c>
       <c r="X41" s="9" t="s">
@@ -28988,7 +28985,7 @@
         <v>0.16034523412527002</v>
       </c>
       <c r="U42">
-        <f t="shared" si="3"/>
+        <f>H42*T42*I42</f>
         <v>0</v>
       </c>
       <c r="X42" s="9" t="s">
@@ -29044,7 +29041,7 @@
       </c>
       <c r="AP42" s="20"/>
       <c r="AQ42" s="18" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="AR42" s="19" t="s">
         <v>117</v>
@@ -29121,7 +29118,7 @@
         <v>0.12642569288891994</v>
       </c>
       <c r="U43">
-        <f t="shared" si="3"/>
+        <f>H43*T43*I43</f>
         <v>230.7268895222789</v>
       </c>
       <c r="X43" s="9" t="s">
@@ -29213,7 +29210,7 @@
     </row>
     <row r="44" spans="5:54" x14ac:dyDescent="0.2">
       <c r="E44" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="F44" t="s">
         <v>119</v>
@@ -29252,7 +29249,7 @@
         <v>0.11191665196287003</v>
       </c>
       <c r="U44">
-        <f t="shared" si="3"/>
+        <f>H44*T44*I44</f>
         <v>408.49577966447561</v>
       </c>
       <c r="X44" s="9" t="s">
@@ -29380,7 +29377,7 @@
         <v>6.4564463903557495E-2</v>
       </c>
       <c r="U45">
-        <f t="shared" si="3"/>
+        <f>H45*T45*I45</f>
         <v>206.20275659198674</v>
       </c>
       <c r="X45" s="9" t="s">
@@ -29508,7 +29505,7 @@
         <v>7.6625966666069981E-2</v>
       </c>
       <c r="U46">
-        <f t="shared" si="3"/>
+        <f>H46*T46*I46</f>
         <v>209.76358374836656</v>
       </c>
       <c r="X46" s="9" t="s">
@@ -29564,7 +29561,7 @@
       </c>
       <c r="AP46" s="20"/>
       <c r="AQ46" s="18" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="AR46" s="19" t="s">
         <v>117</v>
@@ -29641,7 +29638,7 @@
         <v>0.19467496241126997</v>
       </c>
       <c r="U47">
-        <f t="shared" si="3"/>
+        <f>H47*T47*I47</f>
         <v>532.92270960085148</v>
       </c>
       <c r="X47" s="9" t="s">
@@ -29733,7 +29730,7 @@
     </row>
     <row r="48" spans="5:54" x14ac:dyDescent="0.2">
       <c r="E48" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="F48" t="s">
         <v>119</v>
@@ -29772,7 +29769,7 @@
         <v>0.17138540797766999</v>
       </c>
       <c r="U48">
-        <f t="shared" si="3"/>
+        <f>H48*T48*I48</f>
         <v>547.36214672868357</v>
       </c>
       <c r="X48" s="9" t="s">
@@ -29900,7 +29897,7 @@
         <v>0.14782700226492007</v>
       </c>
       <c r="U49">
-        <f t="shared" si="3"/>
+        <f>H49*T49*I49</f>
         <v>269.78427913347912</v>
       </c>
       <c r="X49" s="9" t="s">
@@ -30028,7 +30025,7 @@
         <v>0.16034523412527002</v>
       </c>
       <c r="U50">
-        <f t="shared" si="3"/>
+        <f>H50*T50*I50</f>
         <v>0</v>
       </c>
       <c r="X50" s="9" t="s">
@@ -30084,7 +30081,7 @@
       </c>
       <c r="AP50" s="20"/>
       <c r="AQ50" s="18" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="AR50" s="19" t="s">
         <v>117</v>
@@ -30429,7 +30426,7 @@
       </c>
       <c r="AP54" s="20"/>
       <c r="AQ54" s="18" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AR54" s="19" t="s">
         <v>117</v>
@@ -30780,7 +30777,7 @@
       </c>
       <c r="AP58" s="20"/>
       <c r="AQ58" s="18" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="AR58" s="19" t="s">
         <v>117</v>
@@ -30991,7 +30988,7 @@
         <v>110</v>
       </c>
       <c r="B61" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="C61" t="s">
         <v>113</v>
@@ -31014,36 +31011,39 @@
       <c r="J61">
         <v>0</v>
       </c>
+      <c r="K61">
+        <v>0</v>
+      </c>
       <c r="L61">
         <v>0</v>
       </c>
-      <c r="N61" t="e" cm="1">
-        <f t="array" ref="N61">_xlfn.DROP(_xlfn.XLOOKUP($C61,#REF!,#REF!),1)</f>
-        <v>#REF!</v>
+      <c r="N61" s="32" cm="1">
+        <f t="array" ref="N61:N100">_xlfn.DROP(_xlfn.XLOOKUP($C61,TableW[[#Headers],[ACT/NSW]:[QLD - Low]],TableW[[#All],[ACT/NSW]:[QLD - Low]]),1)</f>
+        <v>80</v>
       </c>
       <c r="P61" cm="1">
         <f t="array" ref="P61:P100">_xlfn.DROP(_xlfn.XLOOKUP($C61,TableLWG[[#Headers],[ACT/NSW]:[QLD - Low]],TableLWG[[#All],[ACT/NSW]:[QLD - Low]]),1)</f>
         <v>0.5</v>
       </c>
       <c r="Q61">
-        <f>(J61 * L61) + (1 - J61 )</f>
-        <v>1</v>
-      </c>
-      <c r="S61" t="e">
+        <f>(J61 * $AD$4 + K61*$AD$5) + (1 - J61 )</f>
+        <v>1</v>
+      </c>
+      <c r="S61">
         <f>(1.185 + 0.00454 * N61- 0.0000026 * N61^2 + 0.315 * P61 )^2 * Q61</f>
-        <v>#REF!</v>
-      </c>
-      <c r="T61" t="e">
+        <v>2.8529236835999998</v>
+      </c>
+      <c r="T61">
         <f>20.7 * S61 * 10^-3</f>
-        <v>#REF!</v>
-      </c>
-      <c r="U61" t="e">
+        <v>5.9055520250520001E-2</v>
+      </c>
+      <c r="U61">
         <f>H61*T61*I61</f>
-        <v>#REF!</v>
-      </c>
-      <c r="V61" t="e">
+        <v>269.44081114299752</v>
+      </c>
+      <c r="V61">
         <f>SUM(U61:U100)/1000</f>
-        <v>#REF!</v>
+        <v>49.157894155502696</v>
       </c>
       <c r="X61" s="9" t="s">
         <v>119</v>
@@ -31142,27 +31142,33 @@
       <c r="J62">
         <v>0</v>
       </c>
+      <c r="K62">
+        <v>0</v>
+      </c>
       <c r="L62">
         <v>0</v>
       </c>
+      <c r="N62">
+        <v>170</v>
+      </c>
       <c r="P62">
         <v>1</v>
       </c>
       <c r="Q62">
-        <f t="shared" ref="Q62:Q100" si="4">(J62 * L62) + (1 - J62 )</f>
+        <f t="shared" ref="Q62:Q100" si="3">(J62 * $AD$4 + K62*$AD$5) + (1 - J62 )</f>
         <v>1</v>
       </c>
       <c r="S62">
-        <f t="shared" ref="S62:S100" si="5">(1.185 + 0.00454 * N62- 0.0000026 * N62^2 + 0.315 * P62 )^2 * Q62</f>
-        <v>2.25</v>
+        <f t="shared" ref="S62:S100" si="4">(1.185 + 0.00454 * N62- 0.0000026 * N62^2 + 0.315 * P62 )^2 * Q62</f>
+        <v>4.8253151556000002</v>
       </c>
       <c r="T62">
-        <f t="shared" ref="T62:T100" si="6">20.7 * S62 * 10^-3</f>
-        <v>4.6574999999999998E-2</v>
+        <f t="shared" ref="T62:T100" si="5">20.7 * S62 * 10^-3</f>
+        <v>9.9884023720920007E-2</v>
       </c>
       <c r="U62">
-        <f t="shared" ref="U62:U100" si="7">H62*T62*I62</f>
-        <v>424.99687499999999</v>
+        <f>H62*T62*I62</f>
+        <v>911.44171645339509</v>
       </c>
       <c r="X62" s="9" t="s">
         <v>120</v>
@@ -31211,7 +31217,7 @@
       </c>
       <c r="AP62" s="20"/>
       <c r="AQ62" s="18" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="AR62" s="19" t="s">
         <v>117</v>
@@ -31260,27 +31266,33 @@
       <c r="J63">
         <v>0</v>
       </c>
+      <c r="K63">
+        <v>0</v>
+      </c>
       <c r="L63">
         <v>0</v>
+      </c>
+      <c r="N63">
+        <v>240</v>
       </c>
       <c r="P63">
         <v>0.8</v>
       </c>
       <c r="Q63">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="S63">
         <f t="shared" si="4"/>
-        <v>1</v>
-      </c>
-      <c r="S63">
+        <v>5.6493683855999981</v>
+      </c>
+      <c r="T63">
         <f t="shared" si="5"/>
-        <v>2.0649690000000001</v>
-      </c>
-      <c r="T63">
-        <f t="shared" si="6"/>
-        <v>4.2744858300000001E-2</v>
+        <v>0.11694192558191996</v>
       </c>
       <c r="U63">
-        <f t="shared" si="7"/>
-        <v>312.03746559000001</v>
+        <f>H63*T63*I63</f>
+        <v>853.67605674801564</v>
       </c>
       <c r="X63" s="9" t="s">
         <v>121</v>
@@ -31376,27 +31388,33 @@
       <c r="J64">
         <v>0</v>
       </c>
+      <c r="K64">
+        <v>0</v>
+      </c>
       <c r="L64">
         <v>0</v>
+      </c>
+      <c r="N64">
+        <v>280</v>
       </c>
       <c r="P64">
         <v>0.4</v>
       </c>
       <c r="Q64">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="S64">
         <f t="shared" si="4"/>
-        <v>1</v>
-      </c>
-      <c r="S64">
+        <v>5.6565962895999995</v>
+      </c>
+      <c r="T64">
         <f t="shared" si="5"/>
-        <v>1.7187209999999999</v>
-      </c>
-      <c r="T64">
-        <f t="shared" si="6"/>
-        <v>3.5577524700000002E-2</v>
+        <v>0.11709154319472</v>
       </c>
       <c r="U64">
-        <f t="shared" si="7"/>
-        <v>227.25143902125001</v>
+        <f>H64*T64*I64</f>
+        <v>747.92223215627394</v>
       </c>
       <c r="AP64" s="20"/>
       <c r="AQ64" s="18"/>
@@ -31450,27 +31468,33 @@
       <c r="J65">
         <v>0</v>
       </c>
+      <c r="K65">
+        <v>0</v>
+      </c>
       <c r="L65">
         <v>0</v>
+      </c>
+      <c r="N65">
+        <v>480</v>
       </c>
       <c r="P65">
         <v>0.2</v>
       </c>
       <c r="Q65">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="S65">
         <f t="shared" si="4"/>
-        <v>1</v>
-      </c>
-      <c r="S65">
+        <v>7.9984889855999999</v>
+      </c>
+      <c r="T65">
         <f t="shared" si="5"/>
-        <v>1.557504</v>
-      </c>
-      <c r="T65">
-        <f t="shared" si="6"/>
-        <v>3.22403328E-2</v>
+        <v>0.16556872200191999</v>
       </c>
       <c r="U65">
-        <f t="shared" si="7"/>
-        <v>58.838607359999997</v>
+        <f>H65*T65*I65</f>
+        <v>302.162917653504</v>
       </c>
       <c r="AP65" s="18"/>
       <c r="AQ65" s="20"/>
@@ -31524,31 +31548,37 @@
       <c r="J66">
         <v>0</v>
       </c>
+      <c r="K66">
+        <v>0</v>
+      </c>
       <c r="L66">
         <v>0</v>
+      </c>
+      <c r="N66">
+        <v>520</v>
       </c>
       <c r="P66">
         <v>0.4</v>
       </c>
       <c r="Q66">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="S66">
         <f t="shared" si="4"/>
-        <v>1</v>
-      </c>
-      <c r="S66">
+        <v>8.8135359375999975</v>
+      </c>
+      <c r="T66">
         <f t="shared" si="5"/>
-        <v>1.7187209999999999</v>
-      </c>
-      <c r="T66">
-        <f t="shared" si="6"/>
-        <v>3.5577524700000002E-2</v>
+        <v>0.18244019390831995</v>
       </c>
       <c r="U66">
-        <f t="shared" si="7"/>
-        <v>259.71593031000003</v>
+        <f>H66*T66*I66</f>
+        <v>1331.8134155307357</v>
       </c>
       <c r="AP66" s="20"/>
       <c r="AQ66" s="18" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="AR66" s="19" t="s">
         <v>117</v>
@@ -31597,27 +31627,33 @@
       <c r="J67">
         <v>0</v>
       </c>
+      <c r="K67">
+        <v>0</v>
+      </c>
       <c r="L67">
         <v>0</v>
+      </c>
+      <c r="N67">
+        <v>550</v>
       </c>
       <c r="P67">
         <v>0.3</v>
       </c>
       <c r="Q67">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="S67">
         <f t="shared" si="4"/>
-        <v>1</v>
-      </c>
-      <c r="S67">
+        <v>8.940100000000001</v>
+      </c>
+      <c r="T67">
         <f t="shared" si="5"/>
-        <v>1.6371202500000002</v>
-      </c>
-      <c r="T67">
-        <f t="shared" si="6"/>
-        <v>3.3888389174999999E-2</v>
+        <v>0.18506007000000002</v>
       </c>
       <c r="U67">
-        <f t="shared" si="7"/>
-        <v>216.46208585531249</v>
+        <f>H67*T67*I67</f>
+        <v>1182.0711971250003</v>
       </c>
       <c r="AP67" s="18"/>
       <c r="AQ67" s="20"/>
@@ -31668,27 +31704,33 @@
       <c r="J68">
         <v>0</v>
       </c>
+      <c r="K68">
+        <v>0</v>
+      </c>
       <c r="L68">
         <v>0</v>
+      </c>
+      <c r="N68">
+        <v>560</v>
       </c>
       <c r="P68">
         <v>0.1</v>
       </c>
       <c r="Q68">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="S68">
         <f t="shared" si="4"/>
-        <v>1</v>
-      </c>
-      <c r="S68">
+        <v>8.6644277315999982</v>
+      </c>
+      <c r="T68">
         <f t="shared" si="5"/>
-        <v>1.4798722500000003</v>
-      </c>
-      <c r="T68">
-        <f t="shared" si="6"/>
-        <v>3.0633355575000007E-2</v>
+        <v>0.17935365404411996</v>
       </c>
       <c r="U68">
-        <f t="shared" si="7"/>
-        <v>167.71762177312505</v>
+        <f>H68*T68*I68</f>
+        <v>981.96125589155668</v>
       </c>
       <c r="AP68" s="20"/>
       <c r="AQ68" s="18"/>
@@ -31742,27 +31784,33 @@
       <c r="J69">
         <v>0</v>
       </c>
+      <c r="K69">
+        <v>0</v>
+      </c>
       <c r="L69">
         <v>0</v>
+      </c>
+      <c r="N69">
+        <v>300</v>
       </c>
       <c r="P69">
         <v>0.4</v>
       </c>
       <c r="Q69">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="S69">
         <f t="shared" si="4"/>
-        <v>1</v>
-      </c>
-      <c r="S69">
+        <v>5.9487209999999981</v>
+      </c>
+      <c r="T69">
         <f t="shared" si="5"/>
-        <v>1.7187209999999999</v>
-      </c>
-      <c r="T69">
-        <f t="shared" si="6"/>
-        <v>3.5577524700000002E-2</v>
+        <v>0.12313852469999996</v>
       </c>
       <c r="U69">
-        <f t="shared" si="7"/>
-        <v>324.64491288750003</v>
+        <f>H69*T69*I69</f>
+        <v>1123.6390378874996</v>
       </c>
       <c r="AP69" s="18"/>
       <c r="AQ69" s="20"/>
@@ -31816,31 +31864,37 @@
       <c r="J70">
         <v>0</v>
       </c>
+      <c r="K70">
+        <v>0</v>
+      </c>
       <c r="L70">
         <v>0</v>
+      </c>
+      <c r="N70">
+        <v>360</v>
       </c>
       <c r="P70">
         <v>0.7</v>
       </c>
       <c r="Q70">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="S70">
         <f t="shared" si="4"/>
-        <v>1</v>
-      </c>
-      <c r="S70">
+        <v>7.3058846435999998</v>
+      </c>
+      <c r="T70">
         <f t="shared" si="5"/>
-        <v>1.9754302499999998</v>
-      </c>
-      <c r="T70">
-        <f t="shared" si="6"/>
-        <v>4.0891406174999992E-2</v>
+        <v>0.15123181212251999</v>
       </c>
       <c r="U70">
-        <f t="shared" si="7"/>
-        <v>671.64134642437489</v>
+        <f>H70*T70*I70</f>
+        <v>2483.9825141123911</v>
       </c>
       <c r="AP70" s="20"/>
       <c r="AQ70" s="18" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="AR70" s="19" t="s">
         <v>117</v>
@@ -31889,27 +31943,33 @@
       <c r="J71">
         <v>0</v>
       </c>
+      <c r="K71">
+        <v>0</v>
+      </c>
       <c r="L71">
         <v>0</v>
+      </c>
+      <c r="N71">
+        <v>390</v>
       </c>
       <c r="P71">
         <v>0.3</v>
       </c>
       <c r="Q71">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="S71">
         <f t="shared" si="4"/>
-        <v>1</v>
-      </c>
-      <c r="S71">
+        <v>7.0471135296000007</v>
+      </c>
+      <c r="T71">
         <f t="shared" si="5"/>
-        <v>1.6371202500000002</v>
-      </c>
-      <c r="T71">
-        <f t="shared" si="6"/>
-        <v>3.3888389174999999E-2</v>
+        <v>0.14587525006272001</v>
       </c>
       <c r="U71">
-        <f t="shared" si="7"/>
-        <v>525.69363707718742</v>
+        <f>H71*T71*I71</f>
+        <v>2262.889816597944</v>
       </c>
       <c r="AP71" s="18"/>
       <c r="AQ71" s="20"/>
@@ -31960,27 +32020,33 @@
       <c r="J72">
         <v>0</v>
       </c>
+      <c r="K72">
+        <v>0</v>
+      </c>
       <c r="L72">
         <v>0</v>
+      </c>
+      <c r="N72">
+        <v>410</v>
       </c>
       <c r="P72">
         <v>0.2</v>
       </c>
       <c r="Q72">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="S72">
         <f t="shared" si="4"/>
-        <v>1</v>
-      </c>
-      <c r="S72">
+        <v>7.1414010756000028</v>
+      </c>
+      <c r="T72">
         <f t="shared" si="5"/>
-        <v>1.557504</v>
-      </c>
-      <c r="T72">
-        <f t="shared" si="6"/>
-        <v>3.22403328E-2</v>
+        <v>0.14782700226492007</v>
       </c>
       <c r="U72">
-        <f t="shared" si="7"/>
-        <v>470.70885887999998</v>
+        <f>H72*T72*I72</f>
+        <v>2158.2742330678329</v>
       </c>
       <c r="AP72" s="20"/>
       <c r="AQ72" s="18"/>
@@ -32034,28 +32100,34 @@
       <c r="J73">
         <v>0.7</v>
       </c>
+      <c r="K73">
+        <v>0</v>
+      </c>
       <c r="L73">
         <f>$AC$12</f>
         <v>1.3</v>
       </c>
+      <c r="N73">
+        <v>440</v>
+      </c>
       <c r="P73">
         <v>0.3</v>
       </c>
       <c r="Q73">
+        <f t="shared" si="3"/>
+        <v>1.21</v>
+      </c>
+      <c r="S73">
         <f t="shared" si="4"/>
-        <v>1.21</v>
-      </c>
-      <c r="S73">
+        <v>9.309296640996001</v>
+      </c>
+      <c r="T73">
         <f t="shared" si="5"/>
-        <v>1.9809155025</v>
-      </c>
-      <c r="T73">
-        <f t="shared" si="6"/>
-        <v>4.1004950901749999E-2</v>
+        <v>0.19270244046861723</v>
       </c>
       <c r="U73">
-        <f t="shared" si="7"/>
-        <v>561.25526546770311</v>
+        <f>H73*T73*I73</f>
+        <v>2637.6146539141982</v>
       </c>
       <c r="AP73" s="18"/>
       <c r="AQ73" s="20"/>
@@ -32109,32 +32181,38 @@
       <c r="J74">
         <v>0</v>
       </c>
+      <c r="K74">
+        <v>0</v>
+      </c>
       <c r="L74">
         <f>$AC$13</f>
         <v>1.1000000000000001</v>
       </c>
+      <c r="N74">
+        <v>470</v>
+      </c>
       <c r="P74">
         <v>0.3</v>
       </c>
       <c r="Q74">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="S74">
         <f t="shared" si="4"/>
-        <v>1</v>
-      </c>
-      <c r="S74">
+        <v>8.0596938816000012</v>
+      </c>
+      <c r="T74">
         <f t="shared" si="5"/>
-        <v>1.6371202500000002</v>
-      </c>
-      <c r="T74">
-        <f t="shared" si="6"/>
-        <v>3.3888389174999999E-2</v>
+        <v>0.16683566334912001</v>
       </c>
       <c r="U74">
-        <f t="shared" si="7"/>
-        <v>773.07887805468749</v>
+        <f>H74*T74*I74</f>
+        <v>3805.9385701518004</v>
       </c>
       <c r="AP74" s="20"/>
       <c r="AQ74" s="18" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="AR74" s="19" t="s">
         <v>117</v>
@@ -32183,28 +32261,34 @@
       <c r="J75">
         <v>0</v>
       </c>
+      <c r="K75">
+        <v>0</v>
+      </c>
       <c r="L75">
         <f>$AC$14</f>
         <v>0</v>
       </c>
+      <c r="N75">
+        <v>490</v>
+      </c>
       <c r="P75">
         <v>0.2</v>
       </c>
       <c r="Q75">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="S75">
         <f t="shared" si="4"/>
-        <v>1</v>
-      </c>
-      <c r="S75">
+        <v>8.1130407556000002</v>
+      </c>
+      <c r="T75">
         <f t="shared" si="5"/>
-        <v>1.557504</v>
-      </c>
-      <c r="T75">
-        <f t="shared" si="6"/>
-        <v>3.22403328E-2</v>
+        <v>0.16793994364092002</v>
       </c>
       <c r="U75">
-        <f t="shared" si="7"/>
-        <v>706.06328831999997</v>
+        <f>H75*T75*I75</f>
+        <v>3677.8847657361484</v>
       </c>
       <c r="AP75" s="18"/>
       <c r="AQ75" s="20"/>
@@ -32255,28 +32339,34 @@
       <c r="J76">
         <v>0.1</v>
       </c>
+      <c r="K76">
+        <v>0</v>
+      </c>
       <c r="L76">
         <f>$AC$14</f>
         <v>0</v>
       </c>
+      <c r="N76">
+        <v>500</v>
+      </c>
       <c r="P76">
         <v>0.1</v>
       </c>
       <c r="Q76">
+        <f t="shared" si="3"/>
+        <v>1.03</v>
+      </c>
+      <c r="S76">
         <f t="shared" si="4"/>
-        <v>0.9</v>
-      </c>
-      <c r="S76">
+        <v>8.2871042175000014</v>
+      </c>
+      <c r="T76">
         <f t="shared" si="5"/>
-        <v>1.3318850250000003</v>
-      </c>
-      <c r="T76">
-        <f t="shared" si="6"/>
-        <v>2.7570020017500006E-2</v>
+        <v>0.17154305730225003</v>
       </c>
       <c r="U76">
-        <f t="shared" si="7"/>
-        <v>503.15286531937511</v>
+        <f>H76*T76*I76</f>
+        <v>3130.6607957660631</v>
       </c>
       <c r="AP76" s="20"/>
       <c r="AQ76" s="18"/>
@@ -32330,28 +32420,34 @@
       <c r="J77">
         <v>0.8</v>
       </c>
+      <c r="K77">
+        <v>0.05</v>
+      </c>
       <c r="L77">
         <f>$AC$12</f>
         <v>1.3</v>
       </c>
+      <c r="N77">
+        <v>75</v>
+      </c>
       <c r="P77">
         <v>0.5</v>
       </c>
       <c r="Q77">
+        <f t="shared" si="3"/>
+        <v>1.2949999999999999</v>
+      </c>
+      <c r="S77">
         <f t="shared" si="4"/>
-        <v>1.24</v>
-      </c>
-      <c r="S77">
+        <v>3.6046003071093744</v>
+      </c>
+      <c r="T77">
         <f t="shared" si="5"/>
-        <v>2.23485975</v>
-      </c>
-      <c r="T77">
-        <f t="shared" si="6"/>
-        <v>4.6261596825000001E-2</v>
+        <v>7.4615226357164055E-2</v>
       </c>
       <c r="U77">
-        <f t="shared" si="7"/>
-        <v>422.13707102812504</v>
+        <f>H77*T77*I77</f>
+        <v>680.86394050912202</v>
       </c>
       <c r="AP77" s="18"/>
       <c r="AQ77" s="20"/>
@@ -32391,7 +32487,7 @@
     </row>
     <row r="78" spans="5:54" x14ac:dyDescent="0.2">
       <c r="E78" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="F78" t="s">
         <v>119</v>
@@ -32404,33 +32500,39 @@
       </c>
       <c r="J78">
         <v>0</v>
+      </c>
+      <c r="K78">
+        <v>0.78</v>
       </c>
       <c r="L78">
         <f>$AC$13</f>
         <v>1.1000000000000001</v>
       </c>
+      <c r="N78">
+        <v>160</v>
+      </c>
       <c r="P78">
         <v>0.9</v>
       </c>
       <c r="Q78">
+        <f t="shared" si="3"/>
+        <v>1.8580000000000001</v>
+      </c>
+      <c r="S78">
         <f t="shared" si="4"/>
-        <v>1</v>
-      </c>
-      <c r="S78">
+        <v>8.4164262871047999</v>
+      </c>
+      <c r="T78">
         <f t="shared" si="5"/>
-        <v>2.1564922500000003</v>
-      </c>
-      <c r="T78">
-        <f t="shared" si="6"/>
-        <v>4.4639389575000001E-2</v>
+        <v>0.17422002414306934</v>
       </c>
       <c r="U78">
-        <f t="shared" si="7"/>
-        <v>773.93541675656252</v>
+        <f>H78*T78*I78</f>
+        <v>3020.5396685804644</v>
       </c>
       <c r="AP78" s="20"/>
       <c r="AQ78" s="18" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="AR78" s="19" t="s">
         <v>117</v>
@@ -32479,28 +32581,34 @@
       <c r="J79">
         <v>0</v>
       </c>
+      <c r="K79">
+        <v>0</v>
+      </c>
       <c r="L79">
         <f>$AC$14</f>
         <v>0</v>
       </c>
+      <c r="N79">
+        <v>220</v>
+      </c>
       <c r="P79">
         <v>0.7</v>
       </c>
       <c r="Q79">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="S79">
         <f t="shared" si="4"/>
-        <v>1</v>
-      </c>
-      <c r="S79">
+        <v>5.1913799715999973</v>
+      </c>
+      <c r="T79">
         <f t="shared" si="5"/>
-        <v>1.9754302499999998</v>
-      </c>
-      <c r="T79">
-        <f t="shared" si="6"/>
-        <v>4.0891406174999992E-2</v>
+        <v>0.10746156541211994</v>
       </c>
       <c r="U79">
-        <f t="shared" si="7"/>
-        <v>727.61145862640603</v>
+        <f>H79*T79*I79</f>
+        <v>1912.1442295519091</v>
       </c>
       <c r="AP79" s="18"/>
       <c r="AQ79" s="20"/>
@@ -32551,28 +32659,34 @@
       <c r="J80">
         <v>0.1</v>
       </c>
+      <c r="K80">
+        <v>0</v>
+      </c>
       <c r="L80">
         <f>$AC$14</f>
         <v>0</v>
       </c>
+      <c r="N80">
+        <v>260</v>
+      </c>
       <c r="P80">
         <v>0.4</v>
       </c>
       <c r="Q80">
+        <f t="shared" si="3"/>
+        <v>1.03</v>
+      </c>
+      <c r="S80">
         <f t="shared" si="4"/>
-        <v>0.9</v>
-      </c>
-      <c r="S80">
+        <v>5.5230542678880008</v>
+      </c>
+      <c r="T80">
         <f t="shared" si="5"/>
-        <v>1.5468489000000001</v>
-      </c>
-      <c r="T80">
-        <f t="shared" si="6"/>
-        <v>3.201977223E-2</v>
+        <v>0.11432722334528161</v>
       </c>
       <c r="U80">
-        <f t="shared" si="7"/>
-        <v>584.3608431975</v>
+        <f>H80*T80*I80</f>
+        <v>2086.4718260513891</v>
       </c>
       <c r="AP80" s="20"/>
       <c r="AQ80" s="18"/>
@@ -32626,28 +32740,34 @@
       <c r="J81">
         <v>0.9</v>
       </c>
+      <c r="K81">
+        <v>0.05</v>
+      </c>
       <c r="L81">
         <f>$AC$12</f>
         <v>1.3</v>
       </c>
+      <c r="N81">
+        <v>440</v>
+      </c>
       <c r="P81">
         <v>0.3</v>
       </c>
       <c r="Q81">
+        <f t="shared" si="3"/>
+        <v>1.3250000000000002</v>
+      </c>
+      <c r="S81">
         <f t="shared" si="4"/>
-        <v>1.27</v>
-      </c>
-      <c r="S81">
+        <v>10.194064503570003</v>
+      </c>
+      <c r="T81">
         <f t="shared" si="5"/>
-        <v>2.0791427175000003</v>
-      </c>
-      <c r="T81">
-        <f t="shared" si="6"/>
-        <v>4.3038254252250004E-2</v>
+        <v>0.21101713522389906</v>
       </c>
       <c r="U81">
-        <f t="shared" si="7"/>
-        <v>196.36203502589063</v>
+        <f>H81*T81*I81</f>
+        <v>962.76567945903957</v>
       </c>
       <c r="AQ81" s="20"/>
       <c r="AR81" s="8" t="s">
@@ -32686,7 +32806,7 @@
     </row>
     <row r="82" spans="5:54" x14ac:dyDescent="0.2">
       <c r="E82" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="F82" t="s">
         <v>119</v>
@@ -32699,29 +32819,35 @@
       </c>
       <c r="J82">
         <v>0</v>
+      </c>
+      <c r="K82">
+        <v>0.9</v>
       </c>
       <c r="L82">
         <f>$AC$13</f>
         <v>1.1000000000000001</v>
       </c>
+      <c r="N82">
+        <v>470</v>
+      </c>
       <c r="P82">
         <v>0.3</v>
       </c>
       <c r="Q82">
+        <f t="shared" si="3"/>
+        <v>1.9900000000000002</v>
+      </c>
+      <c r="S82">
         <f t="shared" si="4"/>
-        <v>1</v>
-      </c>
-      <c r="S82">
+        <v>16.038790824384005</v>
+      </c>
+      <c r="T82">
         <f t="shared" si="5"/>
-        <v>1.6371202500000002</v>
-      </c>
-      <c r="T82">
-        <f t="shared" si="6"/>
-        <v>3.3888389174999999E-2</v>
+        <v>0.33200297006474894</v>
       </c>
       <c r="U82">
-        <f t="shared" si="7"/>
-        <v>309.23155122187495</v>
+        <f>H82*T82*I82</f>
+        <v>3029.5271018408339</v>
       </c>
     </row>
     <row r="83" spans="5:54" x14ac:dyDescent="0.2">
@@ -32737,28 +32863,34 @@
       <c r="J83">
         <v>0</v>
       </c>
+      <c r="K83">
+        <v>0</v>
+      </c>
       <c r="L83">
         <f>$AC$14</f>
         <v>0</v>
       </c>
+      <c r="N83">
+        <v>490</v>
+      </c>
       <c r="P83">
         <v>0.2</v>
       </c>
       <c r="Q83">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="S83">
         <f t="shared" si="4"/>
-        <v>1</v>
-      </c>
-      <c r="S83">
+        <v>8.1130407556000002</v>
+      </c>
+      <c r="T83">
         <f t="shared" si="5"/>
-        <v>1.557504</v>
-      </c>
-      <c r="T83">
-        <f t="shared" si="6"/>
-        <v>3.22403328E-2</v>
+        <v>0.16793994364092002</v>
       </c>
       <c r="U83">
-        <f t="shared" si="7"/>
-        <v>264.77373311999997</v>
+        <f>H83*T83*I83</f>
+        <v>1379.2067871510558</v>
       </c>
     </row>
     <row r="84" spans="5:54" x14ac:dyDescent="0.2">
@@ -32774,28 +32906,34 @@
       <c r="J84">
         <v>0</v>
       </c>
+      <c r="K84">
+        <v>0</v>
+      </c>
       <c r="L84">
         <f>$AC$14</f>
         <v>0</v>
       </c>
+      <c r="N84">
+        <v>500</v>
+      </c>
       <c r="P84">
         <v>0.1</v>
       </c>
       <c r="Q84">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="S84">
         <f t="shared" si="4"/>
-        <v>1</v>
-      </c>
-      <c r="S84">
+        <v>8.0457322500000004</v>
+      </c>
+      <c r="T84">
         <f t="shared" si="5"/>
-        <v>1.4798722500000003</v>
-      </c>
-      <c r="T84">
-        <f t="shared" si="6"/>
-        <v>3.0633355575000007E-2</v>
+        <v>0.16654665757500001</v>
       </c>
       <c r="U84">
-        <f t="shared" si="7"/>
-        <v>223.62349569750006</v>
+        <f>H84*T84*I84</f>
+        <v>1215.7906002975001</v>
       </c>
     </row>
     <row r="85" spans="5:54" x14ac:dyDescent="0.2">
@@ -32814,27 +32952,33 @@
       <c r="J85">
         <v>0</v>
       </c>
+      <c r="K85">
+        <v>0</v>
+      </c>
       <c r="L85">
         <v>0</v>
+      </c>
+      <c r="N85">
+        <v>380</v>
       </c>
       <c r="P85">
         <v>0.4</v>
       </c>
       <c r="Q85">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="S85">
         <f t="shared" si="4"/>
-        <v>1</v>
-      </c>
-      <c r="S85">
+        <v>7.0796437775999967</v>
+      </c>
+      <c r="T85">
         <f t="shared" si="5"/>
-        <v>1.7187209999999999</v>
-      </c>
-      <c r="T85">
-        <f t="shared" si="6"/>
-        <v>3.5577524700000002E-2</v>
+        <v>0.14654862619631992</v>
       </c>
       <c r="U85">
-        <f t="shared" si="7"/>
-        <v>97.393473866250005</v>
+        <f>H85*T85*I85</f>
+        <v>401.17686421242576</v>
       </c>
     </row>
     <row r="86" spans="5:54" x14ac:dyDescent="0.2">
@@ -32853,27 +32997,33 @@
       <c r="J86">
         <v>0</v>
       </c>
+      <c r="K86">
+        <v>0</v>
+      </c>
       <c r="L86">
         <v>0</v>
+      </c>
+      <c r="N86">
+        <v>420</v>
       </c>
       <c r="P86">
         <v>0.4</v>
       </c>
       <c r="Q86">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="S86">
         <f t="shared" si="4"/>
-        <v>1</v>
-      </c>
-      <c r="S86">
+        <v>7.6129639056</v>
+      </c>
+      <c r="T86">
         <f t="shared" si="5"/>
-        <v>1.7187209999999999</v>
-      </c>
-      <c r="T86">
-        <f t="shared" si="6"/>
-        <v>3.5577524700000002E-2</v>
+        <v>0.15758835284591999</v>
       </c>
       <c r="U86">
-        <f t="shared" si="7"/>
-        <v>227.25143902125001</v>
+        <f>H86*T86*I86</f>
+        <v>1006.5956038033139</v>
       </c>
     </row>
     <row r="87" spans="5:54" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -32889,27 +33039,33 @@
       <c r="J87">
         <v>0</v>
       </c>
+      <c r="K87">
+        <v>0</v>
+      </c>
       <c r="L87">
         <v>0</v>
+      </c>
+      <c r="N87">
+        <v>450</v>
       </c>
       <c r="P87">
         <v>0.3</v>
       </c>
       <c r="Q87">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="S87">
         <f t="shared" si="4"/>
-        <v>1</v>
-      </c>
-      <c r="S87">
+        <v>7.8176159999999992</v>
+      </c>
+      <c r="T87">
         <f t="shared" si="5"/>
-        <v>1.6371202500000002</v>
-      </c>
-      <c r="T87">
-        <f t="shared" si="6"/>
-        <v>3.3888389174999999E-2</v>
+        <v>0.16182465119999997</v>
       </c>
       <c r="U87">
-        <f t="shared" si="7"/>
-        <v>123.69262048874999</v>
+        <f>H87*T87*I87</f>
+        <v>590.65997687999993</v>
       </c>
       <c r="AS87" s="2" t="s">
         <v>173</v>
@@ -32955,63 +33111,69 @@
       <c r="J88">
         <v>0</v>
       </c>
+      <c r="K88">
+        <v>0</v>
+      </c>
       <c r="L88">
         <v>0</v>
+      </c>
+      <c r="N88">
+        <v>460</v>
       </c>
       <c r="P88">
         <v>0.1</v>
       </c>
       <c r="Q88">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="S88">
         <f t="shared" si="4"/>
-        <v>1</v>
-      </c>
-      <c r="S88">
+        <v>7.5885924675999998</v>
+      </c>
+      <c r="T88">
         <f t="shared" si="5"/>
-        <v>1.4798722500000003</v>
-      </c>
-      <c r="T88">
-        <f t="shared" si="6"/>
-        <v>3.0633355575000007E-2</v>
+        <v>0.15708386407931998</v>
       </c>
       <c r="U88">
-        <f t="shared" si="7"/>
-        <v>55.905873924375015</v>
+        <f>H88*T88*I88</f>
+        <v>286.67805194475898</v>
       </c>
       <c r="AQ88" s="30" t="s">
+        <v>242</v>
+      </c>
+      <c r="AR88" t="s">
         <v>243</v>
       </c>
-      <c r="AR88" t="s">
+      <c r="AS88" s="2" t="s">
         <v>244</v>
       </c>
-      <c r="AS88" s="2" t="s">
+      <c r="AT88" s="2" t="s">
         <v>245</v>
       </c>
-      <c r="AT88" s="2" t="s">
+      <c r="AU88" s="2" t="s">
         <v>246</v>
       </c>
-      <c r="AU88" s="2" t="s">
+      <c r="AV88" s="3" t="s">
         <v>247</v>
       </c>
-      <c r="AV88" s="3" t="s">
+      <c r="AW88" s="2" t="s">
         <v>248</v>
       </c>
-      <c r="AW88" s="2" t="s">
+      <c r="AX88" s="2" t="s">
         <v>249</v>
       </c>
-      <c r="AX88" s="2" t="s">
+      <c r="AY88" s="2" t="s">
         <v>250</v>
       </c>
-      <c r="AY88" s="2" t="s">
+      <c r="AZ88" s="2" t="s">
         <v>251</v>
       </c>
-      <c r="AZ88" s="2" t="s">
+      <c r="BA88" s="2" t="s">
         <v>252</v>
       </c>
-      <c r="BA88" s="2" t="s">
+      <c r="BB88" s="2" t="s">
         <v>253</v>
-      </c>
-      <c r="BB88" s="2" t="s">
-        <v>254</v>
       </c>
     </row>
     <row r="89" spans="5:54" ht="17" thickTop="1" x14ac:dyDescent="0.2">
@@ -33030,33 +33192,39 @@
       <c r="J89">
         <v>0</v>
       </c>
+      <c r="K89">
+        <v>0</v>
+      </c>
       <c r="L89">
         <v>0</v>
+      </c>
+      <c r="N89">
+        <v>380</v>
       </c>
       <c r="P89">
         <v>0.4</v>
       </c>
       <c r="Q89">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="S89">
         <f t="shared" si="4"/>
-        <v>1</v>
-      </c>
-      <c r="S89">
+        <v>7.0796437775999967</v>
+      </c>
+      <c r="T89">
         <f t="shared" si="5"/>
-        <v>1.7187209999999999</v>
-      </c>
-      <c r="T89">
-        <f t="shared" si="6"/>
-        <v>3.5577524700000002E-2</v>
+        <v>0.14654862619631992</v>
       </c>
       <c r="U89">
-        <f t="shared" si="7"/>
-        <v>97.393473866250005</v>
+        <f>H89*T89*I89</f>
+        <v>401.17686421242576</v>
       </c>
       <c r="X89" t="s">
         <v>130</v>
       </c>
       <c r="Y89" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="Z89" t="s">
         <v>113</v>
@@ -33071,43 +33239,43 @@
         <v>135</v>
       </c>
       <c r="AD89" t="s">
+        <v>255</v>
+      </c>
+      <c r="AE89" t="s">
         <v>256</v>
       </c>
-      <c r="AE89" t="s">
+      <c r="AF89" t="s">
         <v>257</v>
       </c>
-      <c r="AF89" t="s">
+      <c r="AG89" t="s">
         <v>258</v>
       </c>
-      <c r="AG89" t="s">
+      <c r="AH89" t="s">
         <v>259</v>
       </c>
-      <c r="AH89" t="s">
+      <c r="AI89" t="s">
         <v>260</v>
       </c>
-      <c r="AI89" t="s">
+      <c r="AJ89" t="s">
         <v>261</v>
       </c>
-      <c r="AJ89" t="s">
+      <c r="AK89" t="s">
         <v>262</v>
       </c>
-      <c r="AK89" t="s">
+      <c r="AL89" t="s">
         <v>263</v>
       </c>
-      <c r="AL89" t="s">
+      <c r="AM89" t="s">
         <v>264</v>
       </c>
-      <c r="AM89" t="s">
-        <v>265</v>
-      </c>
       <c r="AN89" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="AP89" t="s">
         <v>113</v>
       </c>
       <c r="AQ89" s="30" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="AR89" t="s">
         <v>130</v>
@@ -33145,7 +33313,7 @@
     </row>
     <row r="90" spans="5:54" x14ac:dyDescent="0.2">
       <c r="E90" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="F90" t="s">
         <v>119</v>
@@ -33159,27 +33327,33 @@
       <c r="J90">
         <v>0</v>
       </c>
+      <c r="K90">
+        <v>0</v>
+      </c>
       <c r="L90">
         <v>0</v>
+      </c>
+      <c r="N90">
+        <v>420</v>
       </c>
       <c r="P90">
         <v>0.4</v>
       </c>
       <c r="Q90">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="S90">
         <f t="shared" si="4"/>
-        <v>1</v>
-      </c>
-      <c r="S90">
+        <v>7.6129639056</v>
+      </c>
+      <c r="T90">
         <f t="shared" si="5"/>
-        <v>1.7187209999999999</v>
-      </c>
-      <c r="T90">
-        <f t="shared" si="6"/>
-        <v>3.5577524700000002E-2</v>
+        <v>0.15758835284591999</v>
       </c>
       <c r="U90">
-        <f t="shared" si="7"/>
-        <v>324.64491288750003</v>
+        <f>H90*T90*I90</f>
+        <v>1437.9937197190197</v>
       </c>
       <c r="X90" s="9" t="s">
         <v>117</v>
@@ -33282,27 +33456,33 @@
       <c r="J91">
         <v>0</v>
       </c>
+      <c r="K91">
+        <v>0</v>
+      </c>
       <c r="L91">
         <v>0</v>
+      </c>
+      <c r="N91">
+        <v>450</v>
       </c>
       <c r="P91">
         <v>0.3</v>
       </c>
       <c r="Q91">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="S91">
         <f t="shared" si="4"/>
-        <v>1</v>
-      </c>
-      <c r="S91">
+        <v>7.8176159999999992</v>
+      </c>
+      <c r="T91">
         <f t="shared" si="5"/>
-        <v>1.6371202500000002</v>
-      </c>
-      <c r="T91">
-        <f t="shared" si="6"/>
-        <v>3.3888389174999999E-2</v>
+        <v>0.16182465119999997</v>
       </c>
       <c r="U91">
-        <f t="shared" si="7"/>
-        <v>123.69262048874999</v>
+        <f>H91*T91*I91</f>
+        <v>590.65997687999993</v>
       </c>
       <c r="X91" s="9" t="s">
         <v>119</v>
@@ -33403,26 +33583,32 @@
       <c r="J92">
         <v>0</v>
       </c>
+      <c r="K92">
+        <v>0</v>
+      </c>
       <c r="L92">
         <v>0</v>
+      </c>
+      <c r="N92">
+        <v>460</v>
       </c>
       <c r="P92">
         <v>0.1</v>
       </c>
       <c r="Q92">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="S92">
         <f t="shared" si="4"/>
-        <v>1</v>
-      </c>
-      <c r="S92">
+        <v>7.5885924675999998</v>
+      </c>
+      <c r="T92">
         <f t="shared" si="5"/>
-        <v>1.4798722500000003</v>
-      </c>
-      <c r="T92">
-        <f t="shared" si="6"/>
-        <v>3.0633355575000007E-2</v>
+        <v>0.15708386407931998</v>
       </c>
       <c r="U92">
-        <f t="shared" si="7"/>
+        <f>H92*T92*I92</f>
         <v>0</v>
       </c>
       <c r="X92" s="9" t="s">
@@ -33527,27 +33713,33 @@
       <c r="J93">
         <v>0</v>
       </c>
+      <c r="K93">
+        <v>0</v>
+      </c>
       <c r="L93">
         <v>0</v>
+      </c>
+      <c r="N93">
+        <v>75</v>
       </c>
       <c r="P93">
         <v>0.5</v>
       </c>
       <c r="Q93">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="S93">
         <f t="shared" si="4"/>
-        <v>1</v>
-      </c>
-      <c r="S93">
+        <v>2.7834751406249998</v>
+      </c>
+      <c r="T93">
         <f t="shared" si="5"/>
-        <v>1.80230625</v>
-      </c>
-      <c r="T93">
-        <f t="shared" si="6"/>
-        <v>3.7307739374999996E-2</v>
+        <v>5.7617935410937494E-2</v>
       </c>
       <c r="U93">
-        <f t="shared" si="7"/>
-        <v>68.086624359374994</v>
+        <f>H93*T93*I93</f>
+        <v>105.15273212496092</v>
       </c>
       <c r="X93" s="9" t="s">
         <v>121</v>
@@ -33640,7 +33832,7 @@
     </row>
     <row r="94" spans="5:54" x14ac:dyDescent="0.2">
       <c r="E94" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="F94" t="s">
         <v>119</v>
@@ -33654,27 +33846,33 @@
       <c r="J94">
         <v>0</v>
       </c>
+      <c r="K94">
+        <v>0</v>
+      </c>
       <c r="L94">
         <v>0</v>
+      </c>
+      <c r="N94">
+        <v>160</v>
       </c>
       <c r="P94">
         <v>0.9</v>
       </c>
       <c r="Q94">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="S94">
         <f t="shared" si="4"/>
-        <v>1</v>
-      </c>
-      <c r="S94">
+        <v>4.5298311556000002</v>
+      </c>
+      <c r="T94">
         <f t="shared" si="5"/>
-        <v>2.1564922500000003</v>
-      </c>
-      <c r="T94">
-        <f t="shared" si="6"/>
-        <v>4.4639389575000001E-2</v>
+        <v>9.3767504920920008E-2</v>
       </c>
       <c r="U94">
-        <f t="shared" si="7"/>
-        <v>162.93377194875001</v>
+        <f>H94*T94*I94</f>
+        <v>342.25139296135802</v>
       </c>
       <c r="X94" s="9" t="s">
         <v>117</v>
@@ -33777,27 +33975,33 @@
       <c r="J95">
         <v>0</v>
       </c>
+      <c r="K95">
+        <v>0</v>
+      </c>
       <c r="L95">
         <v>0</v>
+      </c>
+      <c r="N95">
+        <v>220</v>
       </c>
       <c r="P95">
         <v>0.7</v>
       </c>
       <c r="Q95">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="S95">
         <f t="shared" si="4"/>
-        <v>1</v>
-      </c>
-      <c r="S95">
+        <v>5.1913799715999973</v>
+      </c>
+      <c r="T95">
         <f t="shared" si="5"/>
-        <v>1.9754302499999998</v>
-      </c>
-      <c r="T95">
-        <f t="shared" si="6"/>
-        <v>4.0891406174999992E-2</v>
+        <v>0.10746156541211994</v>
       </c>
       <c r="U95">
-        <f t="shared" si="7"/>
-        <v>130.59692847140622</v>
+        <f>H95*T95*I95</f>
+        <v>343.20537453495803</v>
       </c>
       <c r="X95" s="9" t="s">
         <v>119</v>
@@ -33898,27 +34102,33 @@
       <c r="J96">
         <v>0</v>
       </c>
+      <c r="K96">
+        <v>0</v>
+      </c>
       <c r="L96">
         <v>0</v>
+      </c>
+      <c r="N96">
+        <v>260</v>
       </c>
       <c r="P96">
         <v>0.4</v>
       </c>
       <c r="Q96">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="S96">
         <f t="shared" si="4"/>
-        <v>1</v>
-      </c>
-      <c r="S96">
+        <v>5.3621886096000004</v>
+      </c>
+      <c r="T96">
         <f t="shared" si="5"/>
-        <v>1.7187209999999999</v>
-      </c>
-      <c r="T96">
-        <f t="shared" si="6"/>
-        <v>3.5577524700000002E-2</v>
+        <v>0.11099730421872001</v>
       </c>
       <c r="U96">
-        <f t="shared" si="7"/>
-        <v>97.393473866250005</v>
+        <f>H96*T96*I96</f>
+        <v>303.85512029874604</v>
       </c>
       <c r="X96" s="9" t="s">
         <v>120</v>
@@ -34022,27 +34232,33 @@
       <c r="J97">
         <v>0</v>
       </c>
+      <c r="K97">
+        <v>0</v>
+      </c>
       <c r="L97">
         <v>0</v>
+      </c>
+      <c r="N97">
+        <v>380</v>
       </c>
       <c r="P97">
         <v>0.4</v>
       </c>
       <c r="Q97">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="S97">
         <f t="shared" si="4"/>
-        <v>1</v>
-      </c>
-      <c r="S97">
+        <v>7.0796437775999967</v>
+      </c>
+      <c r="T97">
         <f t="shared" si="5"/>
-        <v>1.7187209999999999</v>
-      </c>
-      <c r="T97">
-        <f t="shared" si="6"/>
-        <v>3.5577524700000002E-2</v>
+        <v>0.14654862619631992</v>
       </c>
       <c r="U97">
-        <f t="shared" si="7"/>
-        <v>97.393473866250005</v>
+        <f>H97*T97*I97</f>
+        <v>401.17686421242576</v>
       </c>
       <c r="X97" s="9" t="s">
         <v>121</v>
@@ -34135,7 +34351,7 @@
     </row>
     <row r="98" spans="5:54" x14ac:dyDescent="0.2">
       <c r="E98" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="F98" t="s">
         <v>119</v>
@@ -34149,27 +34365,33 @@
       <c r="J98">
         <v>0</v>
       </c>
+      <c r="K98">
+        <v>0</v>
+      </c>
       <c r="L98">
         <v>0</v>
+      </c>
+      <c r="N98">
+        <v>420</v>
       </c>
       <c r="P98">
         <v>0.4</v>
       </c>
       <c r="Q98">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="S98">
         <f t="shared" si="4"/>
-        <v>1</v>
-      </c>
-      <c r="S98">
+        <v>7.6129639056</v>
+      </c>
+      <c r="T98">
         <f t="shared" si="5"/>
-        <v>1.7187209999999999</v>
-      </c>
-      <c r="T98">
-        <f t="shared" si="6"/>
-        <v>3.5577524700000002E-2</v>
+        <v>0.15758835284591999</v>
       </c>
       <c r="U98">
-        <f t="shared" si="7"/>
-        <v>113.625719510625</v>
+        <f>H98*T98*I98</f>
+        <v>503.29780190165695</v>
       </c>
       <c r="X98" s="9" t="s">
         <v>117</v>
@@ -34272,27 +34494,33 @@
       <c r="J99">
         <v>0</v>
       </c>
+      <c r="K99">
+        <v>0</v>
+      </c>
       <c r="L99">
         <v>0</v>
+      </c>
+      <c r="N99">
+        <v>450</v>
       </c>
       <c r="P99">
         <v>0.3</v>
       </c>
       <c r="Q99">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="S99">
         <f t="shared" si="4"/>
-        <v>1</v>
-      </c>
-      <c r="S99">
+        <v>7.8176159999999992</v>
+      </c>
+      <c r="T99">
         <f t="shared" si="5"/>
-        <v>1.6371202500000002</v>
-      </c>
-      <c r="T99">
-        <f t="shared" si="6"/>
-        <v>3.3888389174999999E-2</v>
+        <v>0.16182465119999997</v>
       </c>
       <c r="U99">
-        <f t="shared" si="7"/>
-        <v>61.846310244374997</v>
+        <f>H99*T99*I99</f>
+        <v>295.32998843999997</v>
       </c>
       <c r="X99" s="9" t="s">
         <v>119</v>
@@ -34393,26 +34621,32 @@
       <c r="J100">
         <v>0</v>
       </c>
+      <c r="K100">
+        <v>0</v>
+      </c>
       <c r="L100">
         <v>0</v>
+      </c>
+      <c r="N100">
+        <v>460</v>
       </c>
       <c r="P100">
         <v>0.1</v>
       </c>
       <c r="Q100">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="S100">
         <f t="shared" si="4"/>
-        <v>1</v>
-      </c>
-      <c r="S100">
+        <v>7.5885924675999998</v>
+      </c>
+      <c r="T100">
         <f t="shared" si="5"/>
-        <v>1.4798722500000003</v>
-      </c>
-      <c r="T100">
-        <f t="shared" si="6"/>
-        <v>3.0633355575000007E-2</v>
+        <v>0.15708386407931998</v>
       </c>
       <c r="U100">
-        <f t="shared" si="7"/>
+        <f>H100*T100*I100</f>
         <v>0</v>
       </c>
       <c r="X100" s="9" t="s">
@@ -34997,7 +35231,7 @@
         <v>1</v>
       </c>
       <c r="AQ106" s="6" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="AR106" s="4" t="s">
         <v>117</v>
@@ -35350,7 +35584,7 @@
         <v>1</v>
       </c>
       <c r="AQ110" s="6" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="AR110" s="4" t="s">
         <v>117</v>
@@ -35703,7 +35937,7 @@
         <v>1</v>
       </c>
       <c r="AQ114" s="6" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="AR114" s="4" t="s">
         <v>117</v>
@@ -36053,7 +36287,7 @@
         <v>1</v>
       </c>
       <c r="AQ118" s="6" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AR118" s="4" t="s">
         <v>117</v>
@@ -36397,7 +36631,7 @@
         <v>1</v>
       </c>
       <c r="AQ122" s="6" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="AR122" s="4" t="s">
         <v>117</v>
@@ -36744,7 +36978,7 @@
         <v>1</v>
       </c>
       <c r="AQ126" s="6" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="AR126" s="4" t="s">
         <v>117</v>
@@ -37028,7 +37262,7 @@
     </row>
     <row r="130" spans="24:54" x14ac:dyDescent="0.2">
       <c r="AQ130" s="6" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="AR130" s="4" t="s">
         <v>117</v>
@@ -37177,7 +37411,7 @@
     </row>
     <row r="134" spans="24:54" x14ac:dyDescent="0.2">
       <c r="AQ134" s="6" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="AR134" s="4" t="s">
         <v>117</v>
@@ -37326,7 +37560,7 @@
     </row>
     <row r="138" spans="24:54" x14ac:dyDescent="0.2">
       <c r="AQ138" s="6" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="AR138" s="4" t="s">
         <v>117</v>
@@ -37475,7 +37709,7 @@
     </row>
     <row r="142" spans="24:54" x14ac:dyDescent="0.2">
       <c r="AQ142" s="6" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="AR142" s="4" t="s">
         <v>117</v>
@@ -37622,7 +37856,7 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="V2:V10 T11 S2:T10 N2:N10 L2:L10 P2:Q10 H2:J10" numberStoredAsText="1"/>
+    <ignoredError sqref="V2:V10 T11 S2:T10 N2:N10 L2:L10 P2:Q10 H2:J9 H10:I10" numberStoredAsText="1"/>
   </ignoredErrors>
   <tableParts count="4">
     <tablePart r:id="rId1"/>
@@ -37647,21 +37881,21 @@
   <sheetData>
     <row r="1" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B1" t="s">
+        <v>291</v>
+      </c>
+      <c r="D1" t="s">
+        <v>289</v>
+      </c>
+      <c r="E1" t="s">
+        <v>292</v>
+      </c>
+      <c r="F1" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="2" spans="2:6" ht="106" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F2" s="33" t="s">
         <v>294</v>
-      </c>
-      <c r="D1" t="s">
-        <v>292</v>
-      </c>
-      <c r="E1" t="s">
-        <v>295</v>
-      </c>
-      <c r="F1" t="s">
-        <v>296</v>
-      </c>
-    </row>
-    <row r="2" spans="2:6" ht="106" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="F2" s="34" t="s">
-        <v>297</v>
       </c>
     </row>
     <row r="3" spans="2:6" x14ac:dyDescent="0.2">
@@ -37669,7 +37903,7 @@
         <v>2025</v>
       </c>
       <c r="C3" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="D3">
         <v>0.1</v>
@@ -37680,7 +37914,7 @@
         <v>2025</v>
       </c>
       <c r="C4" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="D4">
         <v>0.7</v>
@@ -37694,10 +37928,10 @@
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B5" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="C5" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="D5">
         <v>0</v>
@@ -37714,7 +37948,7 @@
         <v>2026</v>
       </c>
       <c r="C6" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="D6">
         <v>0</v>
@@ -37731,7 +37965,7 @@
         <v>2026</v>
       </c>
       <c r="C7" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="D7">
         <v>0.2</v>
@@ -37748,7 +37982,7 @@
         <v>2024</v>
       </c>
       <c r="C12" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="D12">
         <v>0.05</v>
@@ -37763,7 +37997,7 @@
         <v>2024</v>
       </c>
       <c r="C13" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="D13">
         <v>0.05</v>
@@ -37778,7 +38012,7 @@
         <v>2024</v>
       </c>
       <c r="C14" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="D14">
         <v>0.3</v>
@@ -37793,7 +38027,7 @@
         <v>2024</v>
       </c>
       <c r="C15" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="D15">
         <v>0.25</v>
@@ -37808,7 +38042,7 @@
         <v>2024</v>
       </c>
       <c r="C16" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="D16">
         <v>0.15</v>
@@ -37823,7 +38057,7 @@
         <v>2024</v>
       </c>
       <c r="C17" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="D17">
         <v>0</v>
@@ -37838,7 +38072,7 @@
         <v>2025</v>
       </c>
       <c r="C18" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="D18">
         <v>0</v>
@@ -37857,7 +38091,7 @@
         <v>2025</v>
       </c>
       <c r="C19" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="D19">
         <v>0</v>
@@ -37876,7 +38110,7 @@
         <v>2025</v>
       </c>
       <c r="C20" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="D20">
         <v>0</v>
@@ -37895,7 +38129,7 @@
         <v>2025</v>
       </c>
       <c r="C21" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="D21">
         <v>0</v>
@@ -37914,7 +38148,7 @@
         <v>2025</v>
       </c>
       <c r="C22" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="D22">
         <v>0</v>
@@ -37933,7 +38167,7 @@
         <v>2025</v>
       </c>
       <c r="C23" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="D23">
         <v>0</v>
@@ -37952,7 +38186,7 @@
         <v>2025</v>
       </c>
       <c r="C24" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="D24">
         <v>0</v>
@@ -37971,7 +38205,7 @@
         <v>2025</v>
       </c>
       <c r="C25" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="D25">
         <v>0.1</v>
@@ -37990,7 +38224,7 @@
         <v>2025</v>
       </c>
       <c r="C26" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="D26">
         <v>0.2</v>
@@ -38009,7 +38243,7 @@
         <v>2025</v>
       </c>
       <c r="C27" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="D27">
         <v>0.3</v>
@@ -38028,7 +38262,7 @@
         <v>2025</v>
       </c>
       <c r="C28" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="D28">
         <v>0.2</v>
@@ -38047,7 +38281,7 @@
         <v>2025</v>
       </c>
       <c r="C29" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="D29">
         <v>0</v>

</xml_diff>

<commit_message>
test(calculators): adding test case for no calving
</commit_message>
<xml_diff>
--- a/packages/calculators/src/modules/test/3.2-beef-enteric/3.2-beef-enteric.xlsx
+++ b/packages/calculators/src/modules/test/3.2-beef-enteric/3.2-beef-enteric.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eddiesholl/Code/aginnovationaustralia/emissions-calculators/packages/calculators/src/modules/test/3.2-beef-enteric/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:20001_{A9CDA150-C7B8-344A-B152-B20469EC9742}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:20001_{9D25F5B6-DC18-CB45-9AA9-BD7472F19CF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51220" yWindow="14300" windowWidth="28800" windowHeight="28200" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -85,7 +85,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2433" uniqueCount="311">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2434" uniqueCount="313">
   <si>
     <t>EFPRP</t>
   </si>
@@ -1018,6 +1018,12 @@
   </si>
   <si>
     <t>December</t>
+  </si>
+  <si>
+    <t>QLD - Moderate/High - no calving</t>
+  </si>
+  <si>
+    <t>No calving</t>
   </si>
 </sst>
 </file>
@@ -55532,9 +55538,14 @@
         <v>262</v>
       </c>
     </row>
+    <row r="610" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A610" t="s">
+        <v>312</v>
+      </c>
+    </row>
     <row r="611" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A611" t="s">
-        <v>262</v>
+        <v>311</v>
       </c>
       <c r="B611" t="s">
         <v>232</v>
@@ -55592,7 +55603,7 @@
       </c>
       <c r="V611">
         <f>SUM(U611:U650)/1000</f>
-        <v>42.546995304582374</v>
+        <v>41.513791886009763</v>
       </c>
     </row>
     <row r="612" spans="1:22" x14ac:dyDescent="0.2">
@@ -56086,10 +56097,10 @@
         <v>150</v>
       </c>
       <c r="J623">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="K623">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="L623">
         <f>$AC$12</f>
@@ -56103,19 +56114,19 @@
       </c>
       <c r="Q623">
         <f>(J623 * $AD$4 +K623* $AD$5) + (1 -J623 - K623 )</f>
-        <v>1.2150000000000001</v>
+        <v>1</v>
       </c>
       <c r="S623">
         <f t="shared" si="59"/>
-        <v>8.2359239277242935</v>
+        <v>6.7785382121187601</v>
       </c>
       <c r="T623">
         <f t="shared" si="60"/>
-        <v>0.17048362530389286</v>
+        <v>0.14031574099085833</v>
       </c>
       <c r="U623">
         <f>H623*T623*I623</f>
-        <v>2333.4946213470334</v>
+        <v>1920.5717048123736</v>
       </c>
     </row>
     <row r="624" spans="1:22" x14ac:dyDescent="0.2">
@@ -56135,7 +56146,7 @@
         <v>0</v>
       </c>
       <c r="K624">
-        <v>0.71</v>
+        <v>0</v>
       </c>
       <c r="L624">
         <f>$AC$13</f>
@@ -56149,19 +56160,19 @@
       </c>
       <c r="Q624">
         <f t="shared" ref="Q624:Q636" si="61">(J624 * $AD$4 +K624* $AD$5) + (1 -J624 - K624 )</f>
-        <v>1.0710000000000002</v>
+        <v>1</v>
       </c>
       <c r="S624">
         <f t="shared" si="59"/>
-        <v>6.919489694563473</v>
+        <v>6.4607746914691617</v>
       </c>
       <c r="T624">
         <f t="shared" si="60"/>
-        <v>0.14323343667746388</v>
+        <v>0.13373803611341165</v>
       </c>
       <c r="U624">
         <f>H624*T624*I624</f>
-        <v>3267.5127742046448</v>
+        <v>3050.8989488372031</v>
       </c>
     </row>
     <row r="625" spans="5:21" x14ac:dyDescent="0.2">
@@ -56218,7 +56229,7 @@
         <v>200</v>
       </c>
       <c r="J626">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="K626">
         <v>0</v>
@@ -56235,19 +56246,19 @@
       </c>
       <c r="Q626">
         <f t="shared" si="61"/>
-        <v>1.03</v>
+        <v>1</v>
       </c>
       <c r="S626">
         <f t="shared" si="59"/>
-        <v>6.2411086991808444</v>
+        <v>6.0593288341561591</v>
       </c>
       <c r="T626">
         <f t="shared" si="60"/>
-        <v>0.12919095007304346</v>
+        <v>0.12542810686703249</v>
       </c>
       <c r="U626">
         <f>H626*T626*I626</f>
-        <v>2357.7348388330433</v>
+        <v>2289.0629503233426</v>
       </c>
     </row>
     <row r="627" spans="5:21" x14ac:dyDescent="0.2">
@@ -56438,10 +56449,10 @@
         <v>50</v>
       </c>
       <c r="J631">
-        <v>0.9</v>
+        <v>0</v>
       </c>
       <c r="K631">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="L631">
         <f>$AC$12</f>
@@ -56455,19 +56466,19 @@
       </c>
       <c r="Q631">
         <f t="shared" si="61"/>
-        <v>1.2750000000000001</v>
+        <v>1</v>
       </c>
       <c r="S631">
         <f t="shared" si="59"/>
-        <v>9.1459363232214983</v>
+        <v>7.1732833907619584</v>
       </c>
       <c r="T631">
         <f t="shared" si="60"/>
-        <v>0.18932088189068499</v>
+        <v>0.14848696618877252</v>
       </c>
       <c r="U631">
         <f>H631*T631*I631</f>
-        <v>863.77652362625031</v>
+        <v>677.47178323627463</v>
       </c>
     </row>
     <row r="632" spans="5:21" x14ac:dyDescent="0.2">
@@ -56487,7 +56498,7 @@
         <v>0</v>
       </c>
       <c r="K632">
-        <v>0.9</v>
+        <v>0</v>
       </c>
       <c r="L632">
         <f>$AC$13</f>
@@ -56501,19 +56512,19 @@
       </c>
       <c r="Q632">
         <f t="shared" si="61"/>
-        <v>1.0900000000000001</v>
+        <v>1</v>
       </c>
       <c r="S632">
         <f t="shared" si="59"/>
-        <v>9.5337261050566653</v>
+        <v>8.7465377110611602</v>
       </c>
       <c r="T632">
         <f t="shared" si="60"/>
-        <v>0.19734813037467297</v>
+        <v>0.18105333061896603</v>
       </c>
       <c r="U632">
         <f>H632*T632*I632</f>
-        <v>1800.8016896688907</v>
+        <v>1652.111641898065</v>
       </c>
     </row>
     <row r="633" spans="5:21" x14ac:dyDescent="0.2">

</xml_diff>